<commit_message>
1865: revisión de las cifras fijadas por sumas con la copia de Memoria Chilena
La copia de Memoria Chilena confirma 55 de las 62 cifras adoptadas en la pág. 352, las 10 de la
pág. 360 y las del sinóptico (pág. 392). En Itata y Linares (7-15 y 15-25 mujeres) las sumas
admitían dos soluciones; se corrigen 4 cifras según la copia. Quinchao hasta 7 hombres queda
como errata impresa (1336; coherente 1335).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TWJgEkgVBfum8KgacaAb9q
</commit_message>
<xml_diff>
--- a/productos/avance/avance_censos_historicos.xlsx
+++ b/productos/avance/avance_censos_historicos.xlsx
@@ -157,7 +157,7 @@
     <t>Parroquia × sexo × edad (pág. 386, PDF 419) y subdelegación/distrito × sexo × edad desde los bloques provinciales (p. ej. Coquimbo, PDF 302).</t>
   </si>
   <si>
-    <t>Departamento × sexo × edad en 6 tramos (pág. 352) y provincia × sexo × edad (pág. 360) desde la propia publicación; valida 1952 C5 y C6. Departamento (total) desde su sinóptico, validado con el de 1875; provincia × área (1952 C9). Escaneo malo: cifras dudosas fijadas con sumas por fila y por provincia. Errata: Caupolicán 16–25 hombres.</t>
+    <t>Departamento × sexo × edad en 6 tramos (pág. 352) y provincia × sexo × edad (pág. 360) desde la propia publicación; valida 1952 C5 y C6. Departamento (total) desde su sinóptico, validado con el de 1875; provincia × área (1952 C9). Escaneo malo: cifras dudosas fijadas con sumas por fila y por provincia y revisadas con la copia de Memoria Chilena (4 corregidas en Itata y Linares). Erratas: Caupolicán 16–25 hombres y Quinchao hasta 7 hombres.</t>
   </si>
   <si>
     <t>pub_1875</t>
@@ -6433,7 +6433,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:24" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>1865</v>
       </c>
@@ -6513,7 +6513,7 @@
       </c>
       <c r="U9" s="7">
         <f>SUMIFS(Cifras!$J$2:$J$399,Cifras!$A$2:$A$399,$A9)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V9" s="13" t="s">
         <v>40</v>
@@ -7583,7 +7583,7 @@
       </c>
       <c r="U21" s="17">
         <f>SUM(U5:U20)</f>
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.25">
@@ -8681,7 +8681,7 @@
         <v>634</v>
       </c>
       <c r="J31" s="19">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
@@ -50013,7 +50013,7 @@
       </c>
       <c r="M5" s="22">
         <f>SUMIFS(Cifras!$J$2:$J$399,Cifras!$B$2:$B$399,B5,Cifras!$C$2:$C$399,C5)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N5" s="20" t="s">
         <v>1679</v>
@@ -51827,7 +51827,7 @@
       </c>
       <c r="M45" s="23">
         <f>SUM(M2:M44)</f>
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>